<commit_message>
Update soccer trades 2026-07-30 21:03:13 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/Allsvenskan/trades.xlsx
+++ b/data/sxbet/ligas/Allsvenskan/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V2"/>
+  <dimension ref="A1:V3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,102 +531,214 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>0xeddd06e40edd8856b30731382ee5fb74db2f3dbbbc54751058e572781b2ac653</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>21.64</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>1.2163</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Degerfors IF</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Allsvenskan</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>IFK Göteborg vs Degerfors IF</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>IFK Göteborg</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Degerfors IF</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>0x95df1e46a343a30f473be7ab5a70c9f8e18084926552a6d0d301a05441a92e59</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>L19611663</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>1785438282</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>1785672000</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>100.069364</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
           <t>0xde6503f90cec6a47ec5bc8d0a6eea4689c53194f97fad2aebac3314c4e9bbf7b</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>0x86aaA5Ea1D96e252c2C62869556dF1346F9a9264</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr">
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr">
         <is>
           <t>2.24</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>1.4675</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>Asian Handicap (-0.5)</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr">
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr">
         <is>
           <t>Allsvenskan</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>Bk Hacken vs Kalmar FF</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>Bk Hacken</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>Kalmar FF</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t>0xad3b2a98263dca104b4acedfd4bd63e633d2e4f24af4a64ff9bb28a9491fc8c3</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="M3" t="inlineStr">
         <is>
           <t>L19603365</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
+      <c r="N3" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr">
+      <c r="O3" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr">
+      <c r="P3" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr">
+      <c r="Q3" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="R2" t="inlineStr">
+      <c r="R3" t="inlineStr">
         <is>
           <t>1785411359</t>
         </is>
       </c>
-      <c r="S2" t="inlineStr">
+      <c r="S3" t="inlineStr">
         <is>
           <t>1785589200</t>
         </is>
       </c>
-      <c r="T2" t="inlineStr">
+      <c r="T3" t="inlineStr">
         <is>
           <t>4.791444</t>
         </is>
       </c>
-      <c r="U2" t="inlineStr">
+      <c r="U3" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V2" t="inlineStr">
+      <c r="V3" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>

<commit_message>
Update soccer trades 2026-07-31 11:03:33 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/Allsvenskan/trades.xlsx
+++ b/data/sxbet/ligas/Allsvenskan/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V3"/>
+  <dimension ref="A1:V4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,7 +531,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0xeddd06e40edd8856b30731382ee5fb74db2f3dbbbc54751058e572781b2ac653</t>
+          <t>0x35bb1d2972a8c9e91d82c92876853d73d00586e7e2c90b244e71ce4f8e12960f</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -546,22 +546,22 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>21.64</t>
+          <t>22.74</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.2163</t>
+          <t>1.4138</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Asian Handicap (-1)</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Degerfors IF</t>
+          <t>Bk Hacken -1</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -571,27 +571,27 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>IFK Göteborg vs Degerfors IF</t>
+          <t>Bk Hacken vs Kalmar FF</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>IFK Göteborg</t>
+          <t>Bk Hacken</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Degerfors IF</t>
+          <t>Kalmar FF</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0x95df1e46a343a30f473be7ab5a70c9f8e18084926552a6d0d301a05441a92e59</t>
+          <t>0xf0439368071f4ba1f42bafda2c7f19a05013f714bf1536ea251802b6df91ec1b</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>L19611663</t>
+          <t>L19603365</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -616,17 +616,17 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1785438282</t>
+          <t>1785494939</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>1785672000</t>
+          <t>1785589200</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>100.069364</t>
+          <t>54.960725</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -643,102 +643,214 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>0xeddd06e40edd8856b30731382ee5fb74db2f3dbbbc54751058e572781b2ac653</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>21.64</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>1.2163</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Degerfors IF</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Allsvenskan</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>IFK Göteborg vs Degerfors IF</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>IFK Göteborg</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Degerfors IF</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>0x95df1e46a343a30f473be7ab5a70c9f8e18084926552a6d0d301a05441a92e59</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>L19611663</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>1785438282</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>1785672000</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>100.069364</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
           <t>0xde6503f90cec6a47ec5bc8d0a6eea4689c53194f97fad2aebac3314c4e9bbf7b</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>0x86aaA5Ea1D96e252c2C62869556dF1346F9a9264</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr">
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr">
         <is>
           <t>2.24</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>1.4675</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>Asian Handicap (-0.5)</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr">
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr">
         <is>
           <t>Allsvenskan</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>Bk Hacken vs Kalmar FF</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>Bk Hacken</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>Kalmar FF</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t>0xad3b2a98263dca104b4acedfd4bd63e633d2e4f24af4a64ff9bb28a9491fc8c3</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="M4" t="inlineStr">
         <is>
           <t>L19603365</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
+      <c r="N4" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr">
+      <c r="O4" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="P3" t="inlineStr">
+      <c r="P4" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q3" t="inlineStr">
+      <c r="Q4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="R3" t="inlineStr">
+      <c r="R4" t="inlineStr">
         <is>
           <t>1785411359</t>
         </is>
       </c>
-      <c r="S3" t="inlineStr">
+      <c r="S4" t="inlineStr">
         <is>
           <t>1785589200</t>
         </is>
       </c>
-      <c r="T3" t="inlineStr">
+      <c r="T4" t="inlineStr">
         <is>
           <t>4.791444</t>
         </is>
       </c>
-      <c r="U3" t="inlineStr">
+      <c r="U4" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V3" t="inlineStr">
+      <c r="V4" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>

<commit_message>
Update soccer trades 2026-07-31 22:02:27 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/Allsvenskan/trades.xlsx
+++ b/data/sxbet/ligas/Allsvenskan/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V4"/>
+  <dimension ref="A1:V8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,92 +531,84 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0x35bb1d2972a8c9e91d82c92876853d73d00586e7e2c90b244e71ce4f8e12960f</t>
+          <t>0xd43f11093fb4e01c177abb19edf80d9c2efd9bcd10c8449183d688e169b2bce8</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>2.03</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>1.17</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Under/Over (1.5)</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Allsvenskan</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Bk Hacken vs Kalmar FF</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Bk Hacken</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Kalmar FF</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>0x60de0488d91de8628b08a39003f35a0066dbe671648bc58f6f89c95fb9cfb68e</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>L19603365</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>22.74</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>1.4138</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Asian Handicap (-1)</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Bk Hacken -1</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Allsvenskan</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>Bk Hacken vs Kalmar FF</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>Bk Hacken</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>Kalmar FF</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>0xf0439368071f4ba1f42bafda2c7f19a05013f714bf1536ea251802b6df91ec1b</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>L19603365</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>SUCCESS</t>
-        </is>
-      </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1785494939</t>
+          <t>1785534359</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -626,7 +618,7 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>54.960725</t>
+          <t>11.941176</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -643,12 +635,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0xeddd06e40edd8856b30731382ee5fb74db2f3dbbbc54751058e572781b2ac653</t>
+          <t>0x35f6e6f55b350735989f9c70a551b1b492f303f60f6678083396f661c79ea471</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -658,22 +650,22 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>21.64</t>
+          <t>19.02</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.2163</t>
+          <t>1.4138</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Asian Handicap (-1)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Degerfors IF</t>
+          <t>Bk Hacken -1</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -683,27 +675,27 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>IFK Göteborg vs Degerfors IF</t>
+          <t>Bk Hacken vs Kalmar FF</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>IFK Göteborg</t>
+          <t>Bk Hacken</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Degerfors IF</t>
+          <t>Kalmar FF</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>0x95df1e46a343a30f473be7ab5a70c9f8e18084926552a6d0d301a05441a92e59</t>
+          <t>0xf0439368071f4ba1f42bafda2c7f19a05013f714bf1536ea251802b6df91ec1b</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>L19611663</t>
+          <t>L19603365</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -728,17 +720,17 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1785438282</t>
+          <t>1785534359</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>1785672000</t>
+          <t>1785589200</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>100.069364</t>
+          <t>45.969789</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -755,102 +747,550 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>0xd766698e466705ae38c06d2671575880d72ce6bdf5578c2232a0bd68fe1fc381</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>3.80999</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>1.63</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Under/Over (2.5)</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Over 2.5</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Allsvenskan</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Bk Hacken vs Kalmar FF</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Bk Hacken</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Kalmar FF</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>0x375d16e033e4bf094778b7ce9aeabd07dff76d4d30065384ea982ca4aa8eb631</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>L19603365</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>1785533370</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>1785589200</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>6.047603</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>0x5f64f46f8a4871fdf08e07293583bd28a4d596df6764cb46556941dd6d4b7b52</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>5.49</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>1.405</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Under/Over (3.5)</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Over 3.5</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Allsvenskan</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Bk Hacken vs Kalmar FF</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Bk Hacken</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Kalmar FF</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>0xfdddf3a17c3a7b3379814e0885a917a56bc0e70e3d5a5c0b6beddc6ba3dd7921</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>L19603365</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>1785531926</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>1785589200</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>13.555556</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>0x35bb1d2972a8c9e91d82c92876853d73d00586e7e2c90b244e71ce4f8e12960f</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>22.74</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>1.4138</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Asian Handicap (-1)</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Bk Hacken -1</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Allsvenskan</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Bk Hacken vs Kalmar FF</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Bk Hacken</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Kalmar FF</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>0xf0439368071f4ba1f42bafda2c7f19a05013f714bf1536ea251802b6df91ec1b</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>L19603365</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>1785494939</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>1785589200</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>54.960725</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>0xeddd06e40edd8856b30731382ee5fb74db2f3dbbbc54751058e572781b2ac653</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>21.64</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>1.2163</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Degerfors IF</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Allsvenskan</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>IFK Göteborg vs Degerfors IF</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>IFK Göteborg</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Degerfors IF</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>0x95df1e46a343a30f473be7ab5a70c9f8e18084926552a6d0d301a05441a92e59</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>L19611663</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>1785438282</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>1785672000</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>100.069364</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
           <t>0xde6503f90cec6a47ec5bc8d0a6eea4689c53194f97fad2aebac3314c4e9bbf7b</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>0x86aaA5Ea1D96e252c2C62869556dF1346F9a9264</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr">
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="inlineStr">
         <is>
           <t>2.24</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E8" t="inlineStr">
         <is>
           <t>1.4675</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="F8" t="inlineStr">
         <is>
           <t>Asian Handicap (-0.5)</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr">
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr">
         <is>
           <t>Allsvenskan</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="I8" t="inlineStr">
         <is>
           <t>Bk Hacken vs Kalmar FF</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="J8" t="inlineStr">
         <is>
           <t>Bk Hacken</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="K8" t="inlineStr">
         <is>
           <t>Kalmar FF</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="L8" t="inlineStr">
         <is>
           <t>0xad3b2a98263dca104b4acedfd4bd63e633d2e4f24af4a64ff9bb28a9491fc8c3</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="M8" t="inlineStr">
         <is>
           <t>L19603365</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr">
+      <c r="N8" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="O4" t="inlineStr">
+      <c r="O8" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="P4" t="inlineStr">
+      <c r="P8" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q4" t="inlineStr">
+      <c r="Q8" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="R4" t="inlineStr">
+      <c r="R8" t="inlineStr">
         <is>
           <t>1785411359</t>
         </is>
       </c>
-      <c r="S4" t="inlineStr">
+      <c r="S8" t="inlineStr">
         <is>
           <t>1785589200</t>
         </is>
       </c>
-      <c r="T4" t="inlineStr">
+      <c r="T8" t="inlineStr">
         <is>
           <t>4.791444</t>
         </is>
       </c>
-      <c r="U4" t="inlineStr">
+      <c r="U8" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V4" t="inlineStr">
+      <c r="V8" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>

<commit_message>
Update soccer trades 2026-08-01 00:02:51 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/Allsvenskan/trades.xlsx
+++ b/data/sxbet/ligas/Allsvenskan/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V8"/>
+  <dimension ref="A1:V9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,7 +531,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0xd43f11093fb4e01c177abb19edf80d9c2efd9bcd10c8449183d688e169b2bce8</t>
+          <t>0x4b2dea0a5cd4780ebce17ec4dce7e5cf57b818b023f71fcfbd42c674725a80c4</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -542,12 +542,12 @@
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2.03</t>
+          <t>2.99</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.17</t>
+          <t>1.1687</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -608,7 +608,7 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1785534359</t>
+          <t>1785535711</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -618,7 +618,7 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>11.941176</t>
+          <t>17.718519</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -635,89 +635,81 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0x35f6e6f55b350735989f9c70a551b1b492f303f60f6678083396f661c79ea471</t>
+          <t>0xd43f11093fb4e01c177abb19edf80d9c2efd9bcd10c8449183d688e169b2bce8</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>2.03</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>1.17</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Under/Over (1.5)</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Allsvenskan</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Bk Hacken vs Kalmar FF</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Bk Hacken</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Kalmar FF</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>0x60de0488d91de8628b08a39003f35a0066dbe671648bc58f6f89c95fb9cfb68e</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>L19603365</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>19.02</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>1.4138</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Asian Handicap (-1)</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Bk Hacken -1</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Allsvenskan</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>Bk Hacken vs Kalmar FF</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>Bk Hacken</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>Kalmar FF</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>0xf0439368071f4ba1f42bafda2c7f19a05013f714bf1536ea251802b6df91ec1b</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>L19603365</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>SUCCESS</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
       <c r="R3" t="inlineStr">
         <is>
           <t>1785534359</t>
@@ -730,7 +722,7 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>45.969789</t>
+          <t>11.941176</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -747,12 +739,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>0xd766698e466705ae38c06d2671575880d72ce6bdf5578c2232a0bd68fe1fc381</t>
+          <t>0x35f6e6f55b350735989f9c70a551b1b492f303f60f6678083396f661c79ea471</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -762,22 +754,22 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>3.80999</t>
+          <t>19.02</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.63</t>
+          <t>1.4138</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
+          <t>Asian Handicap (-1)</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Over 2.5</t>
+          <t>Bk Hacken -1</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -802,7 +794,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>0x375d16e033e4bf094778b7ce9aeabd07dff76d4d30065384ea982ca4aa8eb631</t>
+          <t>0xf0439368071f4ba1f42bafda2c7f19a05013f714bf1536ea251802b6df91ec1b</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -832,7 +824,7 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>1785533370</t>
+          <t>1785534359</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
@@ -842,7 +834,7 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>6.047603</t>
+          <t>45.969789</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -859,7 +851,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>0x5f64f46f8a4871fdf08e07293583bd28a4d596df6764cb46556941dd6d4b7b52</t>
+          <t>0xd766698e466705ae38c06d2671575880d72ce6bdf5578c2232a0bd68fe1fc381</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -874,22 +866,22 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>5.49</t>
+          <t>3.80999</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.405</t>
+          <t>1.63</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Under/Over (3.5)</t>
+          <t>Under/Over (2.5)</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Over 3.5</t>
+          <t>Over 2.5</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -914,7 +906,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>0xfdddf3a17c3a7b3379814e0885a917a56bc0e70e3d5a5c0b6beddc6ba3dd7921</t>
+          <t>0x375d16e033e4bf094778b7ce9aeabd07dff76d4d30065384ea982ca4aa8eb631</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -944,7 +936,7 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>1785531926</t>
+          <t>1785533370</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
@@ -954,7 +946,7 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>13.555556</t>
+          <t>6.047603</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -971,12 +963,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>0x35bb1d2972a8c9e91d82c92876853d73d00586e7e2c90b244e71ce4f8e12960f</t>
+          <t>0x5f64f46f8a4871fdf08e07293583bd28a4d596df6764cb46556941dd6d4b7b52</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -986,22 +978,22 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>22.74</t>
+          <t>5.49</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1.4138</t>
+          <t>1.405</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
+          <t>Under/Over (3.5)</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Bk Hacken -1</t>
+          <t>Over 3.5</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -1026,7 +1018,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>0xf0439368071f4ba1f42bafda2c7f19a05013f714bf1536ea251802b6df91ec1b</t>
+          <t>0xfdddf3a17c3a7b3379814e0885a917a56bc0e70e3d5a5c0b6beddc6ba3dd7921</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -1056,7 +1048,7 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>1785494939</t>
+          <t>1785531926</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
@@ -1066,7 +1058,7 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>54.960725</t>
+          <t>13.555556</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -1083,7 +1075,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>0xeddd06e40edd8856b30731382ee5fb74db2f3dbbbc54751058e572781b2ac653</t>
+          <t>0x35bb1d2972a8c9e91d82c92876853d73d00586e7e2c90b244e71ce4f8e12960f</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1098,22 +1090,22 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>21.64</t>
+          <t>22.74</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1.2163</t>
+          <t>1.4138</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Asian Handicap (-1)</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Degerfors IF</t>
+          <t>Bk Hacken -1</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -1123,27 +1115,27 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>IFK Göteborg vs Degerfors IF</t>
+          <t>Bk Hacken vs Kalmar FF</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>IFK Göteborg</t>
+          <t>Bk Hacken</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Degerfors IF</t>
+          <t>Kalmar FF</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>0x95df1e46a343a30f473be7ab5a70c9f8e18084926552a6d0d301a05441a92e59</t>
+          <t>0xf0439368071f4ba1f42bafda2c7f19a05013f714bf1536ea251802b6df91ec1b</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>L19611663</t>
+          <t>L19603365</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -1168,17 +1160,17 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>1785438282</t>
+          <t>1785494939</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>1785672000</t>
+          <t>1785589200</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>100.069364</t>
+          <t>54.960725</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1195,102 +1187,214 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>0xeddd06e40edd8856b30731382ee5fb74db2f3dbbbc54751058e572781b2ac653</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>21.64</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>1.2163</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Degerfors IF</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Allsvenskan</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>IFK Göteborg vs Degerfors IF</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>IFK Göteborg</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Degerfors IF</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>0x95df1e46a343a30f473be7ab5a70c9f8e18084926552a6d0d301a05441a92e59</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>L19611663</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>1785438282</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>1785672000</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>100.069364</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
           <t>0xde6503f90cec6a47ec5bc8d0a6eea4689c53194f97fad2aebac3314c4e9bbf7b</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>0x86aaA5Ea1D96e252c2C62869556dF1346F9a9264</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr">
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr">
         <is>
           <t>2.24</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="E9" t="inlineStr">
         <is>
           <t>1.4675</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="F9" t="inlineStr">
         <is>
           <t>Asian Handicap (-0.5)</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr">
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr">
         <is>
           <t>Allsvenskan</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
+      <c r="I9" t="inlineStr">
         <is>
           <t>Bk Hacken vs Kalmar FF</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr">
+      <c r="J9" t="inlineStr">
         <is>
           <t>Bk Hacken</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr">
+      <c r="K9" t="inlineStr">
         <is>
           <t>Kalmar FF</t>
         </is>
       </c>
-      <c r="L8" t="inlineStr">
+      <c r="L9" t="inlineStr">
         <is>
           <t>0xad3b2a98263dca104b4acedfd4bd63e633d2e4f24af4a64ff9bb28a9491fc8c3</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr">
+      <c r="M9" t="inlineStr">
         <is>
           <t>L19603365</t>
         </is>
       </c>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O8" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P8" t="inlineStr">
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q8" t="inlineStr">
+      <c r="Q9" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="R8" t="inlineStr">
+      <c r="R9" t="inlineStr">
         <is>
           <t>1785411359</t>
         </is>
       </c>
-      <c r="S8" t="inlineStr">
+      <c r="S9" t="inlineStr">
         <is>
           <t>1785589200</t>
         </is>
       </c>
-      <c r="T8" t="inlineStr">
+      <c r="T9" t="inlineStr">
         <is>
           <t>4.791444</t>
         </is>
       </c>
-      <c r="U8" t="inlineStr">
+      <c r="U9" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V8" t="inlineStr">
+      <c r="V9" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>